<commit_message>
Dashboard Power BI + ETL combustible clima
</commit_message>
<xml_diff>
--- a/dashboard_combustible_clima.xlsx
+++ b/dashboard_combustible_clima.xlsx
@@ -2818,31 +2818,31 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>16.6</v>
+        <v>13.9</v>
       </c>
       <c r="D2" t="n">
-        <v>15.5</v>
+        <v>13</v>
       </c>
       <c r="E2" t="n">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="F2" t="n">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="G2" t="n">
-        <v>2.2</v>
+        <v>4.9</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Cielo claro</t>
+          <t>Nubes</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-06-07 22:13:29</t>
+          <t>2026-06-09 00:12:02</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -2868,31 +2868,31 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>15.6</v>
+        <v>14.5</v>
       </c>
       <c r="D3" t="n">
-        <v>15.4</v>
+        <v>14.3</v>
       </c>
       <c r="E3" t="n">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="F3" t="n">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="G3" t="n">
-        <v>14.9</v>
+        <v>5.4</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Cielo claro</t>
+          <t>Nubes</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-06-07 22:13:31</t>
+          <t>2026-06-09 00:12:04</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -2918,36 +2918,36 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>8.4</v>
+        <v>11.2</v>
       </c>
       <c r="D4" t="n">
-        <v>8.4</v>
+        <v>10.9</v>
       </c>
       <c r="E4" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F4" t="n">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="G4" t="n">
-        <v>4.3</v>
+        <v>3.4</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Cielo claro</t>
+          <t>Nubes</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-06-07 22:13:33</t>
+          <t>2026-06-09 00:12:06</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Frío (&lt;10°C)</t>
+          <t>Templado (10-20°C)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -2968,31 +2968,31 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>8.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>8.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F5" t="n">
-        <v>1022</v>
+        <v>1015</v>
       </c>
       <c r="G5" t="n">
-        <v>4.5</v>
+        <v>10.9</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Cielo claro</t>
+          <t>Nubes</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-06-07 22:13:35</t>
+          <t>2026-06-09 00:12:08</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -3018,31 +3018,31 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16.4</v>
+        <v>15.5</v>
       </c>
       <c r="D6" t="n">
-        <v>16.3</v>
+        <v>15.2</v>
       </c>
       <c r="E6" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F6" t="n">
-        <v>1016</v>
+        <v>1020</v>
       </c>
       <c r="G6" t="n">
-        <v>6.7</v>
+        <v>0.8</v>
       </c>
       <c r="H6" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Muy nuboso</t>
+          <t>Nubes</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-06-07 22:13:37</t>
+          <t>2026-06-09 00:12:09</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -3541,7 +3541,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>07-06-2026</t>
+          <t>09-06-2026</t>
         </is>
       </c>
     </row>

</xml_diff>